<commit_message>
Generate HTML update history page
</commit_message>
<xml_diff>
--- a/tabiroku-update-history.xlsx
+++ b/tabiroku-update-history.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="運用メモ" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'更新履歴'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'更新履歴'!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -487,32 +487,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:55</t>
+          <t>2026-03-15 14:25</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>702f71e</t>
+          <t>326d02f</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Remove user-facing impact screen</t>
+          <t>Add update history workbook</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>地域価値ダッシュボードを導線から外し、アルバムで完了する流れに変更。</t>
+          <t>更新履歴の CSV / XLSX と、自動生成スクリプトを追加。</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>app.js</t>
+          <t>tabiroku-update-history.csv, tabiroku-update-history.xlsx, tools/export_update_history.py</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>最後がユーザー向けの完了画面として自然になった。</t>
+          <t>更新内容を表形式で共有できるようになった。</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -524,22 +524,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:53</t>
+          <t>2026-03-15 13:55</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4c74fd8</t>
+          <t>702f71e</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Clarify journey recording flow</t>
+          <t>Remove user-facing impact screen</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>旅先ログをトグル記録にし、アルバムへつながる説明文を改善。</t>
+          <t>地域価値ダッシュボードを導線から外し、アルバムで完了する流れに変更。</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>押し間違いを戻しやすく、次の画面も理解しやすくなった。</t>
+          <t>最後がユーザー向けの完了画面として自然になった。</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -561,32 +561,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:50</t>
+          <t>2026-03-15 13:53</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>eb53459</t>
+          <t>4c74fd8</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Refine ask-first mobile flow</t>
+          <t>Clarify journey recording flow</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>おすすめ先行ではなく、相手・したい時間・要望入力から旅提案する流れに変更。</t>
+          <t>旅先ログをトグル記録にし、アルバムへつながる説明文を改善。</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>app.js, styles.css</t>
+          <t>app.js</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>相談してから旅が提案される体験に変わった。</t>
+          <t>押し間違いを戻しやすく、次の画面も理解しやすくなった。</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -598,22 +598,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:42</t>
+          <t>2026-03-15 13:50</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>0cd3250</t>
+          <t>eb53459</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Refine compact screen-first mock</t>
+          <t>Refine ask-first mobile flow</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>iPhone アプリらしい見た目と操作導線になるよう再調整。</t>
+          <t>おすすめ先行ではなく、相手・したい時間・要望入力から旅提案する流れに変更。</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>よりスマホアプリっぽい印象に更新。</t>
+          <t>相談してから旅が提案される体験に変わった。</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -635,22 +635,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:31</t>
+          <t>2026-03-15 12:42</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3ea4570</t>
+          <t>0cd3250</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Compact mobile screens</t>
+          <t>Refine compact screen-first mock</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>余白、文字量、カードの高さを削って画面密度を調整。</t>
+          <t>iPhone アプリらしい見た目と操作導線になるよう再調整。</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>スクロールを減らしたコンパクト UI に改善。</t>
+          <t>よりスマホアプリっぽい印象に更新。</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -672,22 +672,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:23</t>
+          <t>2026-03-15 12:31</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>9516885</t>
+          <t>3ea4570</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Add scenario confirmation step</t>
+          <t>Compact mobile screens</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>旅候補を仮選択してから決定する、2段階の選択操作を追加。</t>
+          <t>余白、文字量、カードの高さを削って画面密度を調整。</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>誤タップしづらい旅選択になった。</t>
+          <t>スクロールを減らしたコンパクト UI に改善。</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -709,32 +709,32 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:19</t>
+          <t>2026-03-15 12:23</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6e43899</t>
+          <t>9516885</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Convert mock to screen-based mobile flow</t>
+          <t>Add scenario confirmation step</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>長い1ページ構成をやめて、画面遷移型のスマホモックへ変更。</t>
+          <t>旅候補を仮選択してから決定する、2段階の選択操作を追加。</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>app.js, index.html, styles.css</t>
+          <t>app.js, styles.css</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>ポチポチ進めるアプリ風の体験に変更。</t>
+          <t>誤タップしづらい旅選択になった。</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -746,32 +746,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:09</t>
+          <t>2026-03-15 12:19</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8417a0a</t>
+          <t>6e43899</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Remove Pages workflow for initial push</t>
+          <t>Convert mock to screen-based mobile flow</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>GitHub Pages の公開方法を workflow からブランチ公開へ切り替えた。</t>
+          <t>長い1ページ構成をやめて、画面遷移型のスマホモックへ変更。</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/pages.yml</t>
+          <t>app.js, index.html, styles.css</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>公開 URL を安定して使える状態に調整。</t>
+          <t>ポチポチ進めるアプリ風の体験に変更。</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -783,32 +783,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:08</t>
+          <t>2026-03-15 12:09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ced69ab</t>
+          <t>8417a0a</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Ignore local GitHub CLI files</t>
+          <t>Remove Pages workflow for initial push</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ローカルの GitHub CLI 関連ファイルを git 管理対象から外した。</t>
+          <t>GitHub Pages の公開方法を workflow からブランチ公開へ切り替えた。</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>.github/workflows/pages.yml</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ユーザー画面の変化なし。</t>
+          <t>公開 URL を安定して使える状態に調整。</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -820,42 +820,79 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>2026-03-15 12:08</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ced69ab</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Ignore local GitHub CLI files</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ローカルの GitHub CLI 関連ファイルを git 管理対象から外した。</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ユーザー画面の変化なし。</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://ryoseiimai.github.io/tabiroku-app/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>2026-03-15 11:33</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>123d0a6</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Initial Tabiroku mobile mock</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>旅録モックの初期画面と、ギフト・旅ログの基本構成を追加。</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>.github/workflows/pages.yml, .gitignore, README.md, app.js</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>最初のスマホモックを確認できる状態に。</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>https://ryoseiimai.github.io/tabiroku-app/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh generated update history
</commit_message>
<xml_diff>
--- a/tabiroku-update-history.xlsx
+++ b/tabiroku-update-history.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="運用メモ" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'更新履歴'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'更新履歴'!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -487,32 +487,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 14:25</t>
+          <t>2026-03-15 14:33</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>326d02f</t>
+          <t>e1cdf24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Add update history workbook</t>
+          <t>Generate HTML update history page</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>更新履歴の CSV / XLSX と、自動生成スクリプトを追加。</t>
+          <t>更新履歴をカード型の HTML ページとして自動生成するようにした。</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>tabiroku-update-history.csv, tabiroku-update-history.xlsx, tools/export_update_history.py</t>
+          <t>README.md, tabiroku-update-history.csv, tabiroku-update-history.xlsx, tools/export_update_history.py</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>更新内容を表形式で共有できるようになった。</t>
+          <t>スプレッドシートより見やすい履歴ページで確認できるようになった。</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -524,32 +524,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:55</t>
+          <t>2026-03-15 14:25</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>702f71e</t>
+          <t>326d02f</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Remove user-facing impact screen</t>
+          <t>Add update history workbook</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>地域価値ダッシュボードを導線から外し、アルバムで完了する流れに変更。</t>
+          <t>更新履歴の CSV / XLSX と、自動生成スクリプトを追加。</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>app.js</t>
+          <t>tabiroku-update-history.csv, tabiroku-update-history.xlsx, tools/export_update_history.py</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>最後がユーザー向けの完了画面として自然になった。</t>
+          <t>更新内容を表形式で共有できるようになった。</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -561,22 +561,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:53</t>
+          <t>2026-03-15 13:55</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>4c74fd8</t>
+          <t>702f71e</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Clarify journey recording flow</t>
+          <t>Remove user-facing impact screen</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>旅先ログをトグル記録にし、アルバムへつながる説明文を改善。</t>
+          <t>地域価値ダッシュボードを導線から外し、アルバムで完了する流れに変更。</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>押し間違いを戻しやすく、次の画面も理解しやすくなった。</t>
+          <t>最後がユーザー向けの完了画面として自然になった。</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -598,32 +598,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 13:50</t>
+          <t>2026-03-15 13:53</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>eb53459</t>
+          <t>4c74fd8</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Refine ask-first mobile flow</t>
+          <t>Clarify journey recording flow</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>おすすめ先行ではなく、相手・したい時間・要望入力から旅提案する流れに変更。</t>
+          <t>旅先ログをトグル記録にし、アルバムへつながる説明文を改善。</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>app.js, styles.css</t>
+          <t>app.js</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>相談してから旅が提案される体験に変わった。</t>
+          <t>押し間違いを戻しやすく、次の画面も理解しやすくなった。</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -635,22 +635,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:42</t>
+          <t>2026-03-15 13:50</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0cd3250</t>
+          <t>eb53459</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Refine compact screen-first mock</t>
+          <t>Refine ask-first mobile flow</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>iPhone アプリらしい見た目と操作導線になるよう再調整。</t>
+          <t>おすすめ先行ではなく、相手・したい時間・要望入力から旅提案する流れに変更。</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>よりスマホアプリっぽい印象に更新。</t>
+          <t>相談してから旅が提案される体験に変わった。</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -672,22 +672,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:31</t>
+          <t>2026-03-15 12:42</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>3ea4570</t>
+          <t>0cd3250</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Compact mobile screens</t>
+          <t>Refine compact screen-first mock</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>余白、文字量、カードの高さを削って画面密度を調整。</t>
+          <t>iPhone アプリらしい見た目と操作導線になるよう再調整。</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>スクロールを減らしたコンパクト UI に改善。</t>
+          <t>よりスマホアプリっぽい印象に更新。</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -709,22 +709,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:23</t>
+          <t>2026-03-15 12:31</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>9516885</t>
+          <t>3ea4570</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Add scenario confirmation step</t>
+          <t>Compact mobile screens</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>旅候補を仮選択してから決定する、2段階の選択操作を追加。</t>
+          <t>余白、文字量、カードの高さを削って画面密度を調整。</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>誤タップしづらい旅選択になった。</t>
+          <t>スクロールを減らしたコンパクト UI に改善。</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -746,32 +746,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:19</t>
+          <t>2026-03-15 12:23</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6e43899</t>
+          <t>9516885</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Convert mock to screen-based mobile flow</t>
+          <t>Add scenario confirmation step</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>長い1ページ構成をやめて、画面遷移型のスマホモックへ変更。</t>
+          <t>旅候補を仮選択してから決定する、2段階の選択操作を追加。</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>app.js, index.html, styles.css</t>
+          <t>app.js, styles.css</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>ポチポチ進めるアプリ風の体験に変更。</t>
+          <t>誤タップしづらい旅選択になった。</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -783,32 +783,32 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:09</t>
+          <t>2026-03-15 12:19</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8417a0a</t>
+          <t>6e43899</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Remove Pages workflow for initial push</t>
+          <t>Convert mock to screen-based mobile flow</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>GitHub Pages の公開方法を workflow からブランチ公開へ切り替えた。</t>
+          <t>長い1ページ構成をやめて、画面遷移型のスマホモックへ変更。</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>.github/workflows/pages.yml</t>
+          <t>app.js, index.html, styles.css</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>公開 URL を安定して使える状態に調整。</t>
+          <t>ポチポチ進めるアプリ風の体験に変更。</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -820,32 +820,32 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-03-15 12:08</t>
+          <t>2026-03-15 12:09</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ced69ab</t>
+          <t>8417a0a</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ignore local GitHub CLI files</t>
+          <t>Remove Pages workflow for initial push</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ローカルの GitHub CLI 関連ファイルを git 管理対象から外した。</t>
+          <t>GitHub Pages の公開方法を workflow からブランチ公開へ切り替えた。</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>.github/workflows/pages.yml</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>ユーザー画面の変化なし。</t>
+          <t>公開 URL を安定して使える状態に調整。</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -857,42 +857,79 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>2026-03-15 12:08</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ced69ab</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Ignore local GitHub CLI files</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ローカルの GitHub CLI 関連ファイルを git 管理対象から外した。</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ユーザー画面の変化なし。</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://ryoseiimai.github.io/tabiroku-app/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>2026-03-15 11:33</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>123d0a6</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Initial Tabiroku mobile mock</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>旅録モックの初期画面と、ギフト・旅ログの基本構成を追加。</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>.github/workflows/pages.yml, .gitignore, README.md, app.js</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>最初のスマホモックを確認できる状態に。</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>https://ryoseiimai.github.io/tabiroku-app/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G12"/>
+  <autoFilter ref="A1:G13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>